<commit_message>
added comments, changes to tc4
</commit_message>
<xml_diff>
--- a/test-data/emiTestData.xlsx
+++ b/test-data/emiTestData.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_29BA46F5A9FA1FB29C3CAB8E12A954EA45547ACC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DB0143B-15AD-40A5-B940-B985C1F8719D}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Tenure Change" state="visible" r:id="rId4"/>
+    <sheet name="Tenure Change" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -43,14 +47,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -413,11 +417,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -453,6 +460,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{e760c494-6550-44b4-8258-77c175d778b7}" enabled="1" method="Privileged" siteId="{76a2ae5a-9f00-4f6b-95ed-5d33d77c4d61}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>